<commit_message>
Įrašyti matmenys, diametras ir suskaičiuoti plotai
</commit_message>
<xml_diff>
--- a/Rezultatai.xlsx
+++ b/Rezultatai.xlsx
@@ -22,7 +22,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -71,7 +73,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -659,25 +663,29 @@
       <c r="D5" s="1" t="n">
         <v>19</v>
       </c>
-      <c r="V5" s="4" t="inlineStr">
-        <is>
-          <t>1,57</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="D6" s="1" t="n">
         <v>58</v>
       </c>
-      <c r="V6" s="4" t="inlineStr">
-        <is>
-          <t>1,75</t>
-        </is>
+      <c r="V6" s="1" t="inlineStr">
+        <is>
+          <t>1,57</t>
+        </is>
+      </c>
+      <c r="W6" s="4">
+        <f>V6*V7</f>
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="D7" s="1" t="n">
         <v>97</v>
+      </c>
+      <c r="V7" s="1" t="inlineStr">
+        <is>
+          <t>1,75</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -1044,13 +1052,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DEBE2C37-2C2D-4C28-A631-0871300752EA}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A133032C-8DA4-4325-99B9-1B63B6280A77}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2CDA3A50-E5E8-4AF6-8F7C-E395BB0529F7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{01AF40AF-96A7-45CC-AFDC-4FF63D6D9469}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90C72CEF-7F82-4BB1-BA65-A03953A50152}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{671E46D8-4263-4B7F-AA57-26D8A7A885B7}"/>
 </file>
</xml_diff>

<commit_message>
sulietis A, B, C stulpeliai pagal matavimo taškų skaičių
</commit_message>
<xml_diff>
--- a/Rezultatai.xlsx
+++ b/Rezultatai.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AH8"/>
+  <dimension ref="A2:AD7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -474,10 +474,6 @@
     <col width="15" customWidth="1" min="28" max="28"/>
     <col width="15" customWidth="1" min="29" max="29"/>
     <col width="15" customWidth="1" min="30" max="30"/>
-    <col width="15" customWidth="1" min="31" max="31"/>
-    <col width="15" customWidth="1" min="32" max="32"/>
-    <col width="15" customWidth="1" min="33" max="33"/>
-    <col width="15" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -525,175 +521,158 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Išmatuotas diferencinis slėgis taškuose 4 linija, Pdi, hPa</t>
+          <t>Pito vamzdelio koeficientas, K</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Išmatuotas diferencinis slėgis taškuose 5 linija, Pdi, hPa</t>
+          <t>Temperatūra ortakyje t, oC</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>Pito vamzdelio koeficientas, K</t>
+          <t>Atmosferinis slėgis P, hPa</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Temperatūra ortakyje t, oC</t>
+          <t>Statinis slėgis ortakyje ± ΔP, hPa</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>Atmosferinis slėgis P, hPa</t>
+          <t>Dujų slėgis kamine Pk= P+ ΔP, hPa</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>Statinis slėgis ortakyje ± ΔP, hPa</t>
+          <t>Dujų mol. masė Ms= qn *22.4, kg/</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>Dujų slėgis kamine Pk= P+ ΔP, hPa</t>
+          <t>Dujų srauto greitis matavimo taškuose, 1 linija, wi = K*129 *√t *√Pdi/ √Pk/√Ms, m/s</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>Dujų mol. masė Ms= qn *22.4, kg/</t>
+          <t>Dujų srauto greitis matavimo taškuose, 2 linija, wi = K*129 *√t *√Pdi/ √Pk/√Ms, m/s</t>
         </is>
       </c>
       <c r="P4" s="3" t="inlineStr">
         <is>
-          <t>Dujų srauto greitis matavimo taškuose, 1 linija, wi = K*129 *√t *√Pdi/ √Pk/√Ms, m/s</t>
+          <t>Dujų srauto greitis matavimo taškuose, 3 linija, wi = K*129 *√t *√Pdi/ √Pk/√Ms, m/s</t>
         </is>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>Dujų srauto greitis matavimo taškuose, 2 linija, wi = K*129 *√t *√Pdi/ √Pk/√Ms, m/s</t>
+          <t>Vidutinis dujų srauto greitis ortakyje w, m/s</t>
         </is>
       </c>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>Dujų srauto greitis matavimo taškuose, 3 linija, wi = K*129 *√t *√Pdi/ √Pk/√Ms, m/s</t>
+          <t>Ortakio diametras, matmenys, m</t>
         </is>
       </c>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t>Dujų srauto greitis matavimo taškuose, 4 linija, wi = K*129 *√t *√Pdi/ √Pk/√Ms, m/s</t>
+          <t>Ortakio skerspjūvio plotas F, m2</t>
         </is>
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>Dujų srauto greitis matavimo taškuose, 5 linija, wi = K*129 *√t *√Pdi/ √Pk/√Ms, m/s</t>
+          <t>Dujų tūrio debitas realiomis sąlygomis Vk = wvid × F, m3/s</t>
         </is>
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
-          <t>Vidutinis dujų srauto greitis ortakyje w, m/s</t>
+          <t>Dujų tūrio debitas normaliosiomis sąlygomis Vdr n.s =Vk *0,269*(P±ΔP)/(273+t), m3/s</t>
         </is>
       </c>
       <c r="V4" s="3" t="inlineStr">
         <is>
-          <t>Ortakio diametras, matmenys, m</t>
+          <t>Vandens kondensato masė m H2O, kg</t>
         </is>
       </c>
       <c r="W4" s="3" t="inlineStr">
         <is>
-          <t>Ortakio skerspjūvio plotas F, m2</t>
+          <t>Vandens garų konc. dujose x=mH2O/Vmn*qn, kg/kg</t>
         </is>
       </c>
       <c r="X4" s="3" t="inlineStr">
         <is>
-          <t>Dujų tūrio debitas realiomis sąlygomis Vk = wvid × F, m3/s</t>
+          <t>Sausų dujų tūrio debitas normaliosiomis sąlygomis Vn= Vdr n.s *((1/(1+(x*qn/0.8038)))</t>
         </is>
       </c>
       <c r="Y4" s="3" t="inlineStr">
         <is>
-          <t>Dujų tūrio debitas normaliosiomis sąlygomis Vdr n.s =Vk *0,269*(P±ΔP)/(273+t), m3/s</t>
+          <t>Prasiurbtas dujų tūris normaliosiomis sąlygomis Vmn, Nm3</t>
         </is>
       </c>
       <c r="Z4" s="3" t="inlineStr">
         <is>
-          <t>Vandens kondensato masė m H2O, kg</t>
+          <t>Išplėstinės neapibrėžties koef. A</t>
         </is>
       </c>
       <c r="AA4" s="3" t="inlineStr">
         <is>
-          <t>Vandens garų konc. dujose x=mH2O/Vmn*qn, kg/kg</t>
+          <t>Išplėstinė neapibrėžtis (dujų tūrio debitas) Uv</t>
         </is>
       </c>
       <c r="AB4" s="3" t="inlineStr">
         <is>
-          <t>Sausų dujų tūrio debitas normaliosiomis sąlygomis Vn= Vdr n.s *((1/(1+(x*qn/0.8038)))</t>
+          <t>Išplėstinė neapibrėžtis (dujų srauto greitis) Uw</t>
         </is>
       </c>
       <c r="AC4" s="3" t="inlineStr">
         <is>
-          <t>Prasiurbtas dujų tūris normaliosiomis sąlygomis Vmn, Nm3</t>
+          <t>Sausų dujų tankis normaliosioms sąlygomis qn, (kg/m3)</t>
         </is>
       </c>
       <c r="AD4" s="3" t="inlineStr">
-        <is>
-          <t>Išplėstinės neapibrėžties koef. A</t>
-        </is>
-      </c>
-      <c r="AE4" s="3" t="inlineStr">
-        <is>
-          <t>Išplėstinė neapibrėžtis (dujų tūrio debitas) Uv</t>
-        </is>
-      </c>
-      <c r="AF4" s="3" t="inlineStr">
-        <is>
-          <t>Išplėstinė neapibrėžtis (dujų srauto greitis) Uw</t>
-        </is>
-      </c>
-      <c r="AG4" s="3" t="inlineStr">
-        <is>
-          <t>Sausų dujų tankis normaliosioms sąlygomis qn, (kg/m3)</t>
-        </is>
-      </c>
-      <c r="AH4" s="3" t="inlineStr">
         <is>
           <t>Skaičiavimus atliko (inicialai, data)</t>
         </is>
       </c>
     </row>
     <row r="5">
+      <c r="A5" s="1" t="n"/>
+      <c r="B5" s="1" t="n"/>
+      <c r="C5" s="1" t="n"/>
       <c r="D5" s="1" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6">
       <c r="D6" s="1" t="n">
-        <v>58</v>
-      </c>
-      <c r="V6" s="1" t="inlineStr">
-        <is>
-          <t>1,57</t>
-        </is>
-      </c>
-      <c r="W6" s="4">
-        <f>V6*V7</f>
+        <v>42.5</v>
+      </c>
+      <c r="R6" s="1" t="inlineStr">
+        <is>
+          <t>0,86</t>
+        </is>
+      </c>
+      <c r="S6" s="4">
+        <f>R6*R7</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="D7" s="1" t="n">
-        <v>97</v>
-      </c>
-      <c r="V7" s="1" t="inlineStr">
-        <is>
-          <t>1,75</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="D8" s="1" t="n">
-        <v>136</v>
+        <v>71</v>
+      </c>
+      <c r="R7" s="1" t="inlineStr">
+        <is>
+          <t>0,87</t>
+        </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="C5:C7"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="B5:B7"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -774,291 +753,4 @@
   <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokumentas" ma:contentTypeID="0x010100BAB57CF81AE55C4698AAD22D302297F0" ma:contentTypeVersion="18" ma:contentTypeDescription="Kurkite naują dokumentą." ma:contentTypeScope="" ma:versionID="49ab401eb4052690d2a2629974c22fd6">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="453e7e53-5eb2-45cf-b2ab-34c867e554b8" xmlns:ns3="aa0d983d-359a-438c-9953-3af1a8ac0831" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ab9969d50e0b13c63bc5bd0499c928dc" ns2:_="" ns3:_="">
-    <xsd:import namespace="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
-    <xsd:import namespace="aa0d983d-359a-438c-9953-3af1a8ac0831"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="453e7e53-5eb2-45cf-b2ab-34c867e554b8" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoTags" ma:index="11" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="12" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="13" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="14" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="15" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceKeyPoints" ma:index="16" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="18" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Vaizdų žymės" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="993cf2ba-b7a7-49f7-97d1-76e12a88c412" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="23" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="24" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="25" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="aa0d983d-359a-438c-9953-3af1a8ac0831" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="19" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{82c4fa3c-500e-4213-91e5-1b9e2014ea63}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="aa0d983d-359a-438c-9953-3af1a8ac0831">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Bendrinama su" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Bendrinta su išsamia informacija" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Turinio tipas"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Antraštė"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="453e7e53-5eb2-45cf-b2ab-34c867e554b8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="aa0d983d-359a-438c-9953-3af1a8ac0831" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A133032C-8DA4-4325-99B9-1B63B6280A77}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{01AF40AF-96A7-45CC-AFDC-4FF63D6D9469}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{671E46D8-4263-4B7F-AA57-26D8A7A885B7}"/>
 </file>
</xml_diff>

<commit_message>
Lapas Greitis perstumtas iš 4 į 5 eilutę
</commit_message>
<xml_diff>
--- a/Rezultatai.xlsx
+++ b/Rezultatai.xlsx
@@ -563,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:Z17"/>
+  <dimension ref="A3:AB12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -592,275 +592,239 @@
     <col width="15" customWidth="1" min="24" max="24"/>
     <col width="15" customWidth="1" min="25" max="25"/>
     <col width="15" customWidth="1" min="26" max="26"/>
+    <col width="15" customWidth="1" min="27" max="27"/>
+    <col width="15" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Debitas pagal matuotą diferencinį slėgį</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="130" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="5" ht="130" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Matavimo data</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Ėminių registracijos Nr. T-107-2026-E-</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Objekto pavadinimas, adresas, taršos šaltinio Nr.</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Matavimo taškai ortakyje nuo vidinės sienelės, cm</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Išmatuotas diferencinis slėgis taškuose 1 linija, Pdi, hPa</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Išmatuotas diferencinis slėgis taškuose 2 linija, Pdi, hPa</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Pito vamzdelio koeficientas, K</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Temperatūra ortakyje t, oC</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Atmosferinis slėgis P, hPa</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>Statinis slėgis ortakyje ± ΔP, hPa</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>Dujų slėgis kamine Pk= P+ ΔP, hPa</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>Dujų mol. masė Ms= qn *22.4, kg/</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>Dujų srauto greitis matavimo taškuose, 1 linija, wi = K*129 *√t *√Pdi/ √Pk/√Ms, m/s</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>Dujų srauto greitis matavimo taškuose, 2 linija, wi = K*129 *√t *√Pdi/ √Pk/√Ms, m/s</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="inlineStr">
         <is>
           <t>Vidutinis dujų srauto greitis ortakyje w, m/s</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="P5" s="3" t="inlineStr">
         <is>
           <t>Ortakio diametras, matmenys, m</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="Q5" s="3" t="inlineStr">
         <is>
           <t>Ortakio skerspjūvio plotas F, m2</t>
         </is>
       </c>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="R5" s="3" t="inlineStr">
         <is>
           <t>Dujų tūrio debitas realiomis sąlygomis Vk = wvid × F, m3/s</t>
         </is>
       </c>
-      <c r="Q4" s="3" t="inlineStr">
+      <c r="S5" s="3" t="inlineStr">
         <is>
           <t>Dujų tūrio debitas normaliosiomis sąlygomis Vdr n.s =Vk *0,269*(P±ΔP)/(273+t), m3/s</t>
         </is>
       </c>
-      <c r="R4" s="3" t="inlineStr">
+      <c r="T5" s="3" t="inlineStr">
         <is>
           <t>Vandens kondensato masė m H2O, kg</t>
         </is>
       </c>
-      <c r="S4" s="3" t="inlineStr">
+      <c r="U5" s="3" t="inlineStr">
         <is>
           <t>Vandens garų konc. dujose x=mH2O/Vmn*qn, kg/kg</t>
         </is>
       </c>
-      <c r="T4" s="3" t="inlineStr">
+      <c r="V5" s="3" t="inlineStr">
         <is>
           <t>Sausų dujų tūrio debitas normaliosiomis sąlygomis Vn= Vdr n.s *((1/(1+(x*qn/0.8038)))</t>
         </is>
       </c>
-      <c r="U4" s="3" t="inlineStr">
+      <c r="W5" s="3" t="inlineStr">
         <is>
           <t>Prasiurbtas dujų tūris normaliosiomis sąlygomis Vmn, Nm3</t>
         </is>
       </c>
-      <c r="V4" s="3" t="inlineStr">
+      <c r="X5" s="3" t="inlineStr">
         <is>
           <t>Išplėstinės neapibrėžties koef. A</t>
         </is>
       </c>
-      <c r="W4" s="3" t="inlineStr">
+      <c r="Y5" s="3" t="inlineStr">
         <is>
           <t>Išplėstinė neapibrėžtis (dujų tūrio debitas) Uv</t>
         </is>
       </c>
-      <c r="X4" s="3" t="inlineStr">
+      <c r="Z5" s="3" t="inlineStr">
         <is>
           <t>Išplėstinė neapibrėžtis (dujų srauto greitis) Uw</t>
         </is>
       </c>
-      <c r="Y4" s="3" t="inlineStr">
+      <c r="AA5" s="3" t="inlineStr">
         <is>
           <t>Sausų dujų tankis normaliosioms sąlygomis qn, (kg/m3)</t>
         </is>
       </c>
-      <c r="Z4" s="3" t="inlineStr">
+      <c r="AB5" s="3" t="inlineStr">
         <is>
           <t>Skaičiavimus atliko (inicialai, data)</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="1" t="n"/>
-      <c r="B5" s="1" t="n"/>
-      <c r="C5" s="1" t="n"/>
-      <c r="D5" s="1" t="n">
+    <row r="6">
+      <c r="A6" s="1" t="n"/>
+      <c r="B6" s="1" t="n"/>
+      <c r="C6" s="1" t="n"/>
+      <c r="D6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="G6" s="6" t="n">
         <v>0.827</v>
       </c>
-      <c r="N5" s="1" t="inlineStr">
+      <c r="P6" s="1" t="inlineStr">
         <is>
           <t>1,20</t>
         </is>
       </c>
-      <c r="O5" s="7">
-        <f>(N5^2*3.14)/4</f>
+      <c r="Q6" s="7">
+        <f>(P6^2*3.14)/4</f>
         <v/>
       </c>
-      <c r="V5" s="6" t="n">
-        <v>0.079</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="D6" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="F6" s="6" t="n">
-        <v>0.827</v>
-      </c>
-      <c r="V6" s="6" t="n">
+      <c r="X6" s="6" t="n">
         <v>0.079</v>
       </c>
     </row>
     <row r="7">
       <c r="D7" s="1" t="n">
-        <v>14</v>
-      </c>
-      <c r="F7" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="G7" s="6" t="n">
         <v>0.827</v>
+      </c>
+      <c r="X7" s="6" t="n">
+        <v>0.079</v>
       </c>
     </row>
     <row r="8">
       <c r="D8" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="F8" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="G8" s="6" t="n">
         <v>0.827</v>
       </c>
     </row>
     <row r="9">
       <c r="D9" s="1" t="n">
-        <v>28</v>
-      </c>
-      <c r="F9" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="G9" s="6" t="n">
         <v>0.827</v>
       </c>
     </row>
     <row r="10">
       <c r="D10" s="1" t="n">
-        <v>39</v>
-      </c>
-      <c r="F10" s="6" t="n">
+        <v>89</v>
+      </c>
+      <c r="G10" s="6" t="n">
         <v>0.827</v>
       </c>
     </row>
     <row r="11">
       <c r="D11" s="1" t="n">
-        <v>60</v>
-      </c>
-      <c r="F11" s="6" t="n">
+        <v>104</v>
+      </c>
+      <c r="G11" s="6" t="n">
         <v>0.827</v>
       </c>
     </row>
     <row r="12">
       <c r="D12" s="1" t="n">
-        <v>81</v>
-      </c>
-      <c r="F12" s="6" t="n">
-        <v>0.827</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="D13" s="1" t="n">
-        <v>92</v>
-      </c>
-      <c r="F13" s="6" t="n">
-        <v>0.827</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="D14" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="F14" s="6" t="n">
-        <v>0.827</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="D15" s="1" t="n">
-        <v>106</v>
-      </c>
-      <c r="F15" s="6" t="n">
-        <v>0.827</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="D16" s="1" t="n">
-        <v>112</v>
-      </c>
-      <c r="F16" s="6" t="n">
-        <v>0.827</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="D17" s="1" t="n">
         <v>115</v>
       </c>
-      <c r="F17" s="6" t="n">
+      <c r="G12" s="6" t="n">
         <v>0.827</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A5:A17"/>
-    <mergeCell ref="B5:B17"/>
-    <mergeCell ref="A2:Z2"/>
-    <mergeCell ref="C5:C17"/>
+    <mergeCell ref="A3:AB3"/>
+    <mergeCell ref="B6:B12"/>
+    <mergeCell ref="C6:C12"/>
+    <mergeCell ref="A6:A12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1121,7 +1085,7 @@
         </is>
       </c>
       <c r="E6" s="10">
-        <f>'Greitis'!O5</f>
+        <f>'Greitis'!Q6</f>
         <v/>
       </c>
     </row>
@@ -1523,23 +1487,25 @@
       <c r="N6" s="16" t="n"/>
       <c r="O6" s="20" t="inlineStr">
         <is>
-          <t>1 linija, 1 filtras</t>
+          <t>2 linijos, 3 filtrai</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="21" t="n"/>
       <c r="B7" s="21" t="n"/>
-      <c r="C7" s="12" t="n"/>
+      <c r="C7" s="17" t="n">
+        <v>2</v>
+      </c>
       <c r="D7" s="21" t="n"/>
-      <c r="E7" s="12" t="n"/>
-      <c r="F7" s="12" t="n"/>
-      <c r="G7" s="12" t="n"/>
+      <c r="E7" s="18" t="n"/>
+      <c r="F7" s="18" t="n"/>
+      <c r="G7" s="18" t="n"/>
       <c r="H7" s="21" t="n"/>
       <c r="I7" s="21" t="n"/>
-      <c r="J7" s="12" t="n"/>
-      <c r="K7" s="12" t="n"/>
-      <c r="L7" s="12" t="n"/>
+      <c r="J7" s="18" t="n"/>
+      <c r="K7" s="18" t="n"/>
+      <c r="L7" s="18" t="n"/>
       <c r="M7" s="19" t="n"/>
       <c r="N7" s="21" t="n"/>
       <c r="O7" s="12" t="n"/>
@@ -1547,16 +1513,18 @@
     <row r="8">
       <c r="A8" s="21" t="n"/>
       <c r="B8" s="21" t="n"/>
-      <c r="C8" s="12" t="n"/>
+      <c r="C8" s="17" t="n">
+        <v>3</v>
+      </c>
       <c r="D8" s="21" t="n"/>
-      <c r="E8" s="12" t="n"/>
-      <c r="F8" s="12" t="n"/>
-      <c r="G8" s="12" t="n"/>
+      <c r="E8" s="18" t="n"/>
+      <c r="F8" s="18" t="n"/>
+      <c r="G8" s="18" t="n"/>
       <c r="H8" s="21" t="n"/>
       <c r="I8" s="21" t="n"/>
-      <c r="J8" s="12" t="n"/>
-      <c r="K8" s="12" t="n"/>
-      <c r="L8" s="12" t="n"/>
+      <c r="J8" s="18" t="n"/>
+      <c r="K8" s="18" t="n"/>
+      <c r="L8" s="18" t="n"/>
       <c r="M8" s="19" t="n"/>
       <c r="N8" s="21" t="n"/>
       <c r="O8" s="12" t="n"/>
@@ -1819,4 +1787,291 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokumentas" ma:contentTypeID="0x010100BAB57CF81AE55C4698AAD22D302297F0" ma:contentTypeVersion="18" ma:contentTypeDescription="Kurkite naują dokumentą." ma:contentTypeScope="" ma:versionID="49ab401eb4052690d2a2629974c22fd6">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="453e7e53-5eb2-45cf-b2ab-34c867e554b8" xmlns:ns3="aa0d983d-359a-438c-9953-3af1a8ac0831" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ab9969d50e0b13c63bc5bd0499c928dc" ns2:_="" ns3:_="">
+    <xsd:import namespace="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
+    <xsd:import namespace="aa0d983d-359a-438c-9953-3af1a8ac0831"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="453e7e53-5eb2-45cf-b2ab-34c867e554b8" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoTags" ma:index="11" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="12" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="13" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="14" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="15" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceKeyPoints" ma:index="16" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="18" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Vaizdų žymės" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="993cf2ba-b7a7-49f7-97d1-76e12a88c412" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="23" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="24" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="25" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="aa0d983d-359a-438c-9953-3af1a8ac0831" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="19" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{82c4fa3c-500e-4213-91e5-1b9e2014ea63}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="aa0d983d-359a-438c-9953-3af1a8ac0831">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Bendrinama su" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Bendrinta su išsamia informacija" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Turinio tipas"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Antraštė"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="453e7e53-5eb2-45cf-b2ab-34c867e554b8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="aa0d983d-359a-438c-9953-3af1a8ac0831" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3D17A693-FB25-430D-B6B5-6C6FA6A677DC}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C6E3F74-698D-4806-8770-263B1DB4FFAE}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3F82DFE4-46CF-46BA-8AA9-D8B27E229D52}"/>
 </file>
</xml_diff>

<commit_message>
Lape Greitis nuspalvota ir nubraižyta lentelė
</commit_message>
<xml_diff>
--- a/Rezultatai.xlsx
+++ b/Rezultatai.xlsx
@@ -43,7 +43,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -60,6 +60,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFFF00"/>
         <bgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF9900"/>
+        <bgColor rgb="00FF9900"/>
       </patternFill>
     </fill>
   </fills>
@@ -222,7 +228,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -272,6 +278,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -666,7 +681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:Z19"/>
+  <dimension ref="A3:Z23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -853,24 +868,34 @@
       <c r="J6" s="18" t="n"/>
       <c r="K6" s="18" t="n"/>
       <c r="L6" s="18" t="n"/>
-      <c r="M6" s="13" t="n"/>
-      <c r="N6" s="1" t="inlineStr">
+      <c r="M6" s="18" t="n"/>
+      <c r="N6" s="15" t="inlineStr">
         <is>
           <t>1,20</t>
         </is>
       </c>
-      <c r="O6" s="7">
+      <c r="O6" s="19">
         <f>(N6^2*3.14)/4</f>
         <v/>
       </c>
-      <c r="V6" s="6" t="n">
+      <c r="P6" s="18" t="n"/>
+      <c r="Q6" s="16" t="n"/>
+      <c r="R6" s="16" t="n"/>
+      <c r="S6" s="18" t="n"/>
+      <c r="T6" s="16" t="n"/>
+      <c r="U6" s="16" t="n"/>
+      <c r="V6" s="17" t="n">
         <v>0.079</v>
       </c>
+      <c r="W6" s="18" t="n"/>
+      <c r="X6" s="18" t="n"/>
+      <c r="Y6" s="16" t="n"/>
+      <c r="Z6" s="13" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="22" t="n"/>
-      <c r="B7" s="22" t="n"/>
-      <c r="C7" s="22" t="n"/>
+      <c r="A7" s="25" t="n"/>
+      <c r="B7" s="25" t="n"/>
+      <c r="C7" s="25" t="n"/>
       <c r="D7" s="15" t="n">
         <v>8</v>
       </c>
@@ -884,14 +909,26 @@
       <c r="J7" s="18" t="n"/>
       <c r="K7" s="18" t="n"/>
       <c r="L7" s="18" t="n"/>
-      <c r="V7" s="6" t="n">
+      <c r="M7" s="13" t="n"/>
+      <c r="N7" s="16" t="n"/>
+      <c r="O7" s="18" t="n"/>
+      <c r="P7" s="18" t="n"/>
+      <c r="Q7" s="16" t="n"/>
+      <c r="R7" s="16" t="n"/>
+      <c r="S7" s="18" t="n"/>
+      <c r="T7" s="16" t="n"/>
+      <c r="U7" s="16" t="n"/>
+      <c r="V7" s="17" t="n">
         <v>0.079</v>
       </c>
+      <c r="W7" s="18" t="n"/>
+      <c r="X7" s="18" t="n"/>
+      <c r="Z7" s="24" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="22" t="n"/>
-      <c r="B8" s="22" t="n"/>
-      <c r="C8" s="22" t="n"/>
+      <c r="A8" s="25" t="n"/>
+      <c r="B8" s="25" t="n"/>
+      <c r="C8" s="25" t="n"/>
       <c r="D8" s="15" t="n">
         <v>14</v>
       </c>
@@ -905,11 +942,16 @@
       <c r="J8" s="18" t="n"/>
       <c r="K8" s="18" t="n"/>
       <c r="L8" s="18" t="n"/>
+      <c r="M8" s="13" t="n"/>
+      <c r="N8" s="16" t="n"/>
+      <c r="O8" s="13" t="n"/>
+      <c r="P8" s="13" t="n"/>
+      <c r="Q8" s="13" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="22" t="n"/>
-      <c r="B9" s="22" t="n"/>
-      <c r="C9" s="22" t="n"/>
+      <c r="A9" s="25" t="n"/>
+      <c r="B9" s="25" t="n"/>
+      <c r="C9" s="25" t="n"/>
       <c r="D9" s="15" t="n">
         <v>20</v>
       </c>
@@ -923,11 +965,16 @@
       <c r="J9" s="18" t="n"/>
       <c r="K9" s="18" t="n"/>
       <c r="L9" s="18" t="n"/>
+      <c r="M9" s="13" t="n"/>
+      <c r="N9" s="13" t="n"/>
+      <c r="O9" s="13" t="n"/>
+      <c r="P9" s="13" t="n"/>
+      <c r="Q9" s="13" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="22" t="n"/>
-      <c r="B10" s="22" t="n"/>
-      <c r="C10" s="22" t="n"/>
+      <c r="A10" s="25" t="n"/>
+      <c r="B10" s="25" t="n"/>
+      <c r="C10" s="25" t="n"/>
       <c r="D10" s="15" t="n">
         <v>28</v>
       </c>
@@ -943,9 +990,9 @@
       <c r="L10" s="18" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="22" t="n"/>
-      <c r="B11" s="22" t="n"/>
-      <c r="C11" s="22" t="n"/>
+      <c r="A11" s="25" t="n"/>
+      <c r="B11" s="25" t="n"/>
+      <c r="C11" s="25" t="n"/>
       <c r="D11" s="15" t="n">
         <v>39</v>
       </c>
@@ -961,9 +1008,9 @@
       <c r="L11" s="18" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="22" t="n"/>
-      <c r="B12" s="22" t="n"/>
-      <c r="C12" s="22" t="n"/>
+      <c r="A12" s="25" t="n"/>
+      <c r="B12" s="25" t="n"/>
+      <c r="C12" s="25" t="n"/>
       <c r="D12" s="15" t="n">
         <v>60</v>
       </c>
@@ -979,9 +1026,9 @@
       <c r="L12" s="18" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="22" t="n"/>
-      <c r="B13" s="22" t="n"/>
-      <c r="C13" s="22" t="n"/>
+      <c r="A13" s="25" t="n"/>
+      <c r="B13" s="25" t="n"/>
+      <c r="C13" s="25" t="n"/>
       <c r="D13" s="15" t="n">
         <v>81</v>
       </c>
@@ -997,9 +1044,9 @@
       <c r="L13" s="18" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="22" t="n"/>
-      <c r="B14" s="22" t="n"/>
-      <c r="C14" s="22" t="n"/>
+      <c r="A14" s="25" t="n"/>
+      <c r="B14" s="25" t="n"/>
+      <c r="C14" s="25" t="n"/>
       <c r="D14" s="15" t="n">
         <v>92</v>
       </c>
@@ -1015,9 +1062,9 @@
       <c r="L14" s="18" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="22" t="n"/>
-      <c r="B15" s="22" t="n"/>
-      <c r="C15" s="22" t="n"/>
+      <c r="A15" s="25" t="n"/>
+      <c r="B15" s="25" t="n"/>
+      <c r="C15" s="25" t="n"/>
       <c r="D15" s="15" t="n">
         <v>100</v>
       </c>
@@ -1033,9 +1080,9 @@
       <c r="L15" s="18" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="22" t="n"/>
-      <c r="B16" s="22" t="n"/>
-      <c r="C16" s="22" t="n"/>
+      <c r="A16" s="25" t="n"/>
+      <c r="B16" s="25" t="n"/>
+      <c r="C16" s="25" t="n"/>
       <c r="D16" s="15" t="n">
         <v>106</v>
       </c>
@@ -1051,9 +1098,9 @@
       <c r="L16" s="18" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="22" t="n"/>
-      <c r="B17" s="22" t="n"/>
-      <c r="C17" s="22" t="n"/>
+      <c r="A17" s="25" t="n"/>
+      <c r="B17" s="25" t="n"/>
+      <c r="C17" s="25" t="n"/>
       <c r="D17" s="15" t="n">
         <v>112</v>
       </c>
@@ -1069,9 +1116,9 @@
       <c r="L17" s="18" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="21" t="n"/>
-      <c r="B18" s="21" t="n"/>
-      <c r="C18" s="21" t="n"/>
+      <c r="A18" s="24" t="n"/>
+      <c r="B18" s="24" t="n"/>
+      <c r="C18" s="24" t="n"/>
       <c r="D18" s="15" t="n">
         <v>115</v>
       </c>
@@ -1088,13 +1135,63 @@
     </row>
     <row r="19">
       <c r="A19" s="13" t="n"/>
+      <c r="B19" s="13" t="n"/>
+      <c r="C19" s="13" t="n"/>
+      <c r="D19" s="13" t="n"/>
+      <c r="E19" s="13" t="n"/>
+      <c r="F19" s="13" t="n"/>
+      <c r="G19" s="13" t="n"/>
+      <c r="H19" s="13" t="n"/>
+      <c r="I19" s="13" t="n"/>
+      <c r="J19" s="13" t="n"/>
+      <c r="K19" s="13" t="n"/>
+      <c r="L19" s="13" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="n"/>
+      <c r="B20" s="13" t="n"/>
+      <c r="C20" s="13" t="n"/>
+      <c r="D20" s="20" t="inlineStr">
+        <is>
+          <t>RPU***</t>
+        </is>
+      </c>
+      <c r="E20" s="21" t="inlineStr">
+        <is>
+          <t>Kai bus 2 linijos, RPU*** yra 2 linijos vidurinis taškas</t>
+        </is>
+      </c>
+      <c r="F20" s="22" t="n"/>
+      <c r="G20" s="22" t="n"/>
+      <c r="H20" s="22" t="n"/>
+      <c r="I20" s="22" t="n"/>
+      <c r="J20" s="22" t="n"/>
+      <c r="K20" s="22" t="n"/>
+      <c r="L20" s="23" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="n"/>
+      <c r="B21" s="13" t="n"/>
+      <c r="C21" s="13" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="n"/>
+      <c r="B22" s="13" t="n"/>
+      <c r="C22" s="13" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="n"/>
+      <c r="B23" s="13" t="n"/>
+      <c r="C23" s="13" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
+    <mergeCell ref="E20:L20"/>
+    <mergeCell ref="A3:Z3"/>
     <mergeCell ref="B6:B18"/>
-    <mergeCell ref="A3:Z3"/>
     <mergeCell ref="C6:C18"/>
     <mergeCell ref="A6:A18"/>
+    <mergeCell ref="Z6:Z7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1622,68 +1719,68 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="n"/>
-      <c r="B6" s="23" t="n"/>
-      <c r="C6" s="24" t="n"/>
-      <c r="D6" s="25" t="n"/>
-      <c r="E6" s="26" t="n"/>
-      <c r="F6" s="26" t="n"/>
-      <c r="G6" s="26" t="n"/>
-      <c r="H6" s="26" t="n"/>
-      <c r="I6" s="26" t="n"/>
-      <c r="J6" s="26" t="n"/>
-      <c r="K6" s="26" t="n"/>
-      <c r="L6" s="27" t="n"/>
-      <c r="M6" s="27" t="n"/>
-      <c r="N6" s="24" t="n"/>
-      <c r="O6" s="24" t="n">
+      <c r="A6" s="26" t="n"/>
+      <c r="B6" s="26" t="n"/>
+      <c r="C6" s="27" t="n"/>
+      <c r="D6" s="28" t="n"/>
+      <c r="E6" s="29" t="n"/>
+      <c r="F6" s="29" t="n"/>
+      <c r="G6" s="29" t="n"/>
+      <c r="H6" s="29" t="n"/>
+      <c r="I6" s="29" t="n"/>
+      <c r="J6" s="29" t="n"/>
+      <c r="K6" s="29" t="n"/>
+      <c r="L6" s="30" t="n"/>
+      <c r="M6" s="30" t="n"/>
+      <c r="N6" s="27" t="n"/>
+      <c r="O6" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="P6" s="28" t="inlineStr">
+      <c r="P6" s="31" t="inlineStr">
         <is>
           <t>1 linija, 1 filtras</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="29" t="n"/>
-      <c r="B7" s="29" t="n"/>
-      <c r="C7" s="31" t="n"/>
-      <c r="D7" s="25" t="n"/>
-      <c r="E7" s="26" t="n"/>
-      <c r="F7" s="26" t="n"/>
-      <c r="G7" s="26" t="n"/>
-      <c r="H7" s="26" t="n"/>
-      <c r="I7" s="26" t="n"/>
-      <c r="J7" s="26" t="n"/>
-      <c r="K7" s="26" t="n"/>
-      <c r="L7" s="31" t="n"/>
-      <c r="M7" s="31" t="n"/>
-      <c r="N7" s="31" t="n"/>
-      <c r="O7" s="31" t="n"/>
-      <c r="P7" s="28" t="inlineStr">
+      <c r="A7" s="32" t="n"/>
+      <c r="B7" s="32" t="n"/>
+      <c r="C7" s="34" t="n"/>
+      <c r="D7" s="28" t="n"/>
+      <c r="E7" s="29" t="n"/>
+      <c r="F7" s="29" t="n"/>
+      <c r="G7" s="29" t="n"/>
+      <c r="H7" s="29" t="n"/>
+      <c r="I7" s="29" t="n"/>
+      <c r="J7" s="29" t="n"/>
+      <c r="K7" s="29" t="n"/>
+      <c r="L7" s="34" t="n"/>
+      <c r="M7" s="34" t="n"/>
+      <c r="N7" s="34" t="n"/>
+      <c r="O7" s="34" t="n"/>
+      <c r="P7" s="31" t="inlineStr">
         <is>
           <t>1 linija, 2 filtras</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="30" t="n"/>
-      <c r="B8" s="30" t="n"/>
-      <c r="C8" s="32" t="n"/>
-      <c r="D8" s="25" t="n"/>
-      <c r="E8" s="26" t="n"/>
-      <c r="F8" s="26" t="n"/>
-      <c r="G8" s="26" t="n"/>
-      <c r="H8" s="26" t="n"/>
-      <c r="I8" s="26" t="n"/>
-      <c r="J8" s="26" t="n"/>
-      <c r="K8" s="26" t="n"/>
-      <c r="L8" s="32" t="n"/>
-      <c r="M8" s="32" t="n"/>
-      <c r="N8" s="32" t="n"/>
-      <c r="O8" s="32" t="n"/>
-      <c r="P8" s="25" t="n"/>
+      <c r="A8" s="33" t="n"/>
+      <c r="B8" s="33" t="n"/>
+      <c r="C8" s="35" t="n"/>
+      <c r="D8" s="28" t="n"/>
+      <c r="E8" s="29" t="n"/>
+      <c r="F8" s="29" t="n"/>
+      <c r="G8" s="29" t="n"/>
+      <c r="H8" s="29" t="n"/>
+      <c r="I8" s="29" t="n"/>
+      <c r="J8" s="29" t="n"/>
+      <c r="K8" s="29" t="n"/>
+      <c r="L8" s="35" t="n"/>
+      <c r="M8" s="35" t="n"/>
+      <c r="N8" s="35" t="n"/>
+      <c r="O8" s="35" t="n"/>
+      <c r="P8" s="28" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1757,8 +1854,8 @@
           <t>Filtro/indo svoris prieš KD ėmimą mpr (g)</t>
         </is>
       </c>
-      <c r="F4" s="19" t="n"/>
-      <c r="G4" s="20" t="n"/>
+      <c r="F4" s="22" t="n"/>
+      <c r="G4" s="23" t="n"/>
       <c r="H4" s="12" t="inlineStr">
         <is>
           <t>Atsakingo asmens inicialai, data</t>
@@ -1774,8 +1871,8 @@
           <t>Filtro/indo svoris po KD ėmimo mpo (g)</t>
         </is>
       </c>
-      <c r="K4" s="19" t="n"/>
-      <c r="L4" s="20" t="n"/>
+      <c r="K4" s="22" t="n"/>
+      <c r="L4" s="23" t="n"/>
       <c r="M4" s="12" t="inlineStr">
         <is>
           <t>Kietųjų dalelių svoris mf/Svorių pokytis (g) (&lt;2,20 g filtro talpumas)</t>
@@ -1793,10 +1890,10 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="n"/>
-      <c r="B5" s="21" t="n"/>
-      <c r="C5" s="21" t="n"/>
-      <c r="D5" s="21" t="n"/>
+      <c r="A5" s="24" t="n"/>
+      <c r="B5" s="24" t="n"/>
+      <c r="C5" s="24" t="n"/>
+      <c r="D5" s="24" t="n"/>
       <c r="E5" s="12" t="inlineStr">
         <is>
           <t>1</t>
@@ -1812,8 +1909,8 @@
           <t>3</t>
         </is>
       </c>
-      <c r="H5" s="21" t="n"/>
-      <c r="I5" s="21" t="n"/>
+      <c r="H5" s="24" t="n"/>
+      <c r="I5" s="24" t="n"/>
       <c r="J5" s="12" t="inlineStr">
         <is>
           <t>1</t>
@@ -1829,252 +1926,252 @@
           <t>3</t>
         </is>
       </c>
-      <c r="M5" s="21" t="n"/>
-      <c r="N5" s="21" t="n"/>
-      <c r="O5" s="21" t="n"/>
+      <c r="M5" s="24" t="n"/>
+      <c r="N5" s="24" t="n"/>
+      <c r="O5" s="24" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="33" t="n"/>
-      <c r="B6" s="33" t="n"/>
+      <c r="A6" s="36" t="n"/>
+      <c r="B6" s="36" t="n"/>
       <c r="C6" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="33" t="n"/>
+      <c r="D6" s="36" t="n"/>
       <c r="E6" s="16" t="n"/>
       <c r="F6" s="16" t="n"/>
       <c r="G6" s="16" t="n"/>
-      <c r="H6" s="33" t="n"/>
-      <c r="I6" s="33" t="n"/>
+      <c r="H6" s="36" t="n"/>
+      <c r="I6" s="36" t="n"/>
       <c r="J6" s="16" t="n"/>
       <c r="K6" s="16" t="n"/>
       <c r="L6" s="16" t="n"/>
       <c r="M6" s="18" t="n"/>
-      <c r="N6" s="33" t="n"/>
-      <c r="O6" s="34" t="inlineStr">
+      <c r="N6" s="36" t="n"/>
+      <c r="O6" s="37" t="inlineStr">
         <is>
           <t>1 linija, 2 filtrai</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="35" t="n"/>
-      <c r="B7" s="35" t="n"/>
+      <c r="A7" s="38" t="n"/>
+      <c r="B7" s="38" t="n"/>
       <c r="C7" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="35" t="n"/>
+      <c r="D7" s="38" t="n"/>
       <c r="E7" s="16" t="n"/>
       <c r="F7" s="16" t="n"/>
       <c r="G7" s="16" t="n"/>
-      <c r="H7" s="35" t="n"/>
-      <c r="I7" s="35" t="n"/>
+      <c r="H7" s="38" t="n"/>
+      <c r="I7" s="38" t="n"/>
       <c r="J7" s="16" t="n"/>
       <c r="K7" s="16" t="n"/>
       <c r="L7" s="16" t="n"/>
       <c r="M7" s="18" t="n"/>
-      <c r="N7" s="35" t="n"/>
+      <c r="N7" s="38" t="n"/>
       <c r="O7" s="13" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="35" t="n"/>
-      <c r="B8" s="35" t="n"/>
+      <c r="A8" s="38" t="n"/>
+      <c r="B8" s="38" t="n"/>
       <c r="C8" s="13" t="n"/>
-      <c r="D8" s="35" t="n"/>
+      <c r="D8" s="38" t="n"/>
       <c r="E8" s="13" t="n"/>
       <c r="F8" s="13" t="n"/>
       <c r="G8" s="13" t="n"/>
-      <c r="H8" s="35" t="n"/>
-      <c r="I8" s="35" t="n"/>
+      <c r="H8" s="38" t="n"/>
+      <c r="I8" s="38" t="n"/>
       <c r="J8" s="13" t="n"/>
       <c r="K8" s="13" t="n"/>
       <c r="L8" s="13" t="n"/>
       <c r="M8" s="18" t="n"/>
-      <c r="N8" s="35" t="n"/>
+      <c r="N8" s="38" t="n"/>
       <c r="O8" s="13" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="35" t="n"/>
-      <c r="B9" s="35" t="n"/>
+      <c r="A9" s="38" t="n"/>
+      <c r="B9" s="38" t="n"/>
       <c r="C9" s="14" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D9" s="35" t="n"/>
+      <c r="D9" s="38" t="n"/>
       <c r="E9" s="16" t="n"/>
       <c r="F9" s="16" t="n"/>
       <c r="G9" s="16" t="n"/>
-      <c r="H9" s="35" t="n"/>
-      <c r="I9" s="35" t="n"/>
+      <c r="H9" s="38" t="n"/>
+      <c r="I9" s="38" t="n"/>
       <c r="J9" s="16" t="n"/>
       <c r="K9" s="16" t="n"/>
       <c r="L9" s="16" t="n"/>
       <c r="M9" s="18" t="n"/>
-      <c r="N9" s="35" t="n"/>
-      <c r="O9" s="36" t="inlineStr">
+      <c r="N9" s="38" t="n"/>
+      <c r="O9" s="39" t="inlineStr">
         <is>
           <t>Tuščiasis ėminys (mt)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="35" t="n"/>
-      <c r="B10" s="35" t="n"/>
+      <c r="A10" s="38" t="n"/>
+      <c r="B10" s="38" t="n"/>
       <c r="C10" s="13" t="n"/>
-      <c r="D10" s="35" t="n"/>
+      <c r="D10" s="38" t="n"/>
       <c r="E10" s="13" t="n"/>
       <c r="F10" s="13" t="n"/>
       <c r="G10" s="13" t="n"/>
-      <c r="H10" s="35" t="n"/>
-      <c r="I10" s="35" t="n"/>
+      <c r="H10" s="38" t="n"/>
+      <c r="I10" s="38" t="n"/>
       <c r="J10" s="13" t="n"/>
       <c r="K10" s="13" t="n"/>
       <c r="L10" s="13" t="n"/>
       <c r="M10" s="13" t="n"/>
-      <c r="N10" s="35" t="n"/>
+      <c r="N10" s="38" t="n"/>
       <c r="O10" s="13" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="35" t="n"/>
-      <c r="B11" s="35" t="n"/>
+      <c r="A11" s="38" t="n"/>
+      <c r="B11" s="38" t="n"/>
       <c r="C11" s="14" t="inlineStr">
         <is>
           <t>41</t>
         </is>
       </c>
-      <c r="D11" s="35" t="n"/>
+      <c r="D11" s="38" t="n"/>
       <c r="E11" s="16" t="n"/>
       <c r="F11" s="16" t="n"/>
       <c r="G11" s="16" t="n"/>
-      <c r="H11" s="35" t="n"/>
-      <c r="I11" s="35" t="n"/>
+      <c r="H11" s="38" t="n"/>
+      <c r="I11" s="38" t="n"/>
       <c r="J11" s="16" t="n"/>
       <c r="K11" s="16" t="n"/>
       <c r="L11" s="16" t="n"/>
       <c r="M11" s="18" t="n"/>
-      <c r="N11" s="35" t="n"/>
-      <c r="O11" s="36" t="inlineStr">
+      <c r="N11" s="38" t="n"/>
+      <c r="O11" s="39" t="inlineStr">
         <is>
           <t>Išplautos nuosėdos (mn)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="35" t="n"/>
-      <c r="B12" s="35" t="n"/>
+      <c r="A12" s="38" t="n"/>
+      <c r="B12" s="38" t="n"/>
       <c r="C12" s="14" t="inlineStr">
         <is>
           <t>00</t>
         </is>
       </c>
-      <c r="D12" s="35" t="n"/>
+      <c r="D12" s="38" t="n"/>
       <c r="E12" s="16" t="n"/>
       <c r="F12" s="16" t="n"/>
       <c r="G12" s="16" t="n"/>
-      <c r="H12" s="35" t="n"/>
-      <c r="I12" s="35" t="n"/>
+      <c r="H12" s="38" t="n"/>
+      <c r="I12" s="38" t="n"/>
       <c r="J12" s="16" t="n"/>
       <c r="K12" s="16" t="n"/>
       <c r="L12" s="16" t="n"/>
       <c r="M12" s="18" t="n"/>
-      <c r="N12" s="35" t="n"/>
-      <c r="O12" s="36" t="inlineStr">
+      <c r="N12" s="38" t="n"/>
+      <c r="O12" s="39" t="inlineStr">
         <is>
           <t>Išvalytos ėminių sistemos tuščiasis ėminys (mIt)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="35" t="n"/>
-      <c r="B13" s="35" t="n"/>
+      <c r="A13" s="38" t="n"/>
+      <c r="B13" s="38" t="n"/>
       <c r="C13" s="14" t="inlineStr">
         <is>
           <t>01</t>
         </is>
       </c>
-      <c r="D13" s="35" t="n"/>
+      <c r="D13" s="38" t="n"/>
       <c r="E13" s="16" t="n"/>
       <c r="F13" s="16" t="n"/>
       <c r="G13" s="16" t="n"/>
-      <c r="H13" s="35" t="n"/>
-      <c r="I13" s="35" t="n"/>
+      <c r="H13" s="38" t="n"/>
+      <c r="I13" s="38" t="n"/>
       <c r="J13" s="16" t="n"/>
       <c r="K13" s="16" t="n"/>
       <c r="L13" s="16" t="n"/>
       <c r="M13" s="18" t="n"/>
-      <c r="N13" s="35" t="n"/>
-      <c r="O13" s="36" t="inlineStr">
+      <c r="N13" s="38" t="n"/>
+      <c r="O13" s="39" t="inlineStr">
         <is>
           <t>Tušti indai svorio kontrolei (mIt1)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="35" t="n"/>
-      <c r="B14" s="35" t="n"/>
+      <c r="A14" s="38" t="n"/>
+      <c r="B14" s="38" t="n"/>
       <c r="C14" s="14" t="inlineStr">
         <is>
           <t>02</t>
         </is>
       </c>
-      <c r="D14" s="35" t="n"/>
+      <c r="D14" s="38" t="n"/>
       <c r="E14" s="16" t="n"/>
       <c r="F14" s="16" t="n"/>
       <c r="G14" s="16" t="n"/>
-      <c r="H14" s="35" t="n"/>
-      <c r="I14" s="35" t="n"/>
+      <c r="H14" s="38" t="n"/>
+      <c r="I14" s="38" t="n"/>
       <c r="J14" s="16" t="n"/>
       <c r="K14" s="16" t="n"/>
       <c r="L14" s="16" t="n"/>
       <c r="M14" s="18" t="n"/>
-      <c r="N14" s="35" t="n"/>
-      <c r="O14" s="36" t="inlineStr">
+      <c r="N14" s="38" t="n"/>
+      <c r="O14" s="39" t="inlineStr">
         <is>
           <t>Tušti indai svorio kontrolei (mIt2)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="35" t="n"/>
-      <c r="B15" s="35" t="n"/>
+      <c r="A15" s="38" t="n"/>
+      <c r="B15" s="38" t="n"/>
       <c r="C15" s="14" t="inlineStr">
         <is>
           <t>03</t>
         </is>
       </c>
-      <c r="D15" s="35" t="n"/>
+      <c r="D15" s="38" t="n"/>
       <c r="E15" s="16" t="n"/>
       <c r="F15" s="16" t="n"/>
       <c r="G15" s="16" t="n"/>
-      <c r="H15" s="35" t="n"/>
-      <c r="I15" s="35" t="n"/>
+      <c r="H15" s="38" t="n"/>
+      <c r="I15" s="38" t="n"/>
       <c r="J15" s="16" t="n"/>
       <c r="K15" s="16" t="n"/>
       <c r="L15" s="16" t="n"/>
       <c r="M15" s="18" t="n"/>
-      <c r="N15" s="35" t="n"/>
-      <c r="O15" s="36" t="inlineStr">
+      <c r="N15" s="38" t="n"/>
+      <c r="O15" s="39" t="inlineStr">
         <is>
           <t>Tušti indai svorio kontrolei (mIt3)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="37" t="n"/>
-      <c r="B16" s="37" t="n"/>
+      <c r="A16" s="40" t="n"/>
+      <c r="B16" s="40" t="n"/>
       <c r="C16" s="13" t="n"/>
-      <c r="D16" s="37" t="n"/>
+      <c r="D16" s="40" t="n"/>
       <c r="E16" s="13" t="n"/>
       <c r="F16" s="13" t="n"/>
       <c r="G16" s="13" t="n"/>
-      <c r="H16" s="37" t="n"/>
-      <c r="I16" s="37" t="n"/>
+      <c r="H16" s="40" t="n"/>
+      <c r="I16" s="40" t="n"/>
       <c r="J16" s="13" t="n"/>
       <c r="K16" s="13" t="n"/>
       <c r="L16" s="13" t="n"/>
       <c r="M16" s="18" t="n"/>
-      <c r="N16" s="37" t="n"/>
-      <c r="O16" s="36" t="inlineStr">
+      <c r="N16" s="40" t="n"/>
+      <c r="O16" s="39" t="inlineStr">
         <is>
           <t>Tuščių indų ir išvalytos ėminių sistemos tuščiojo ėminio svorio pokytis (mItp)</t>
         </is>
@@ -2150,4 +2247,291 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokumentas" ma:contentTypeID="0x010100BAB57CF81AE55C4698AAD22D302297F0" ma:contentTypeVersion="18" ma:contentTypeDescription="Kurkite naują dokumentą." ma:contentTypeScope="" ma:versionID="49ab401eb4052690d2a2629974c22fd6">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="453e7e53-5eb2-45cf-b2ab-34c867e554b8" xmlns:ns3="aa0d983d-359a-438c-9953-3af1a8ac0831" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ab9969d50e0b13c63bc5bd0499c928dc" ns2:_="" ns3:_="">
+    <xsd:import namespace="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
+    <xsd:import namespace="aa0d983d-359a-438c-9953-3af1a8ac0831"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="453e7e53-5eb2-45cf-b2ab-34c867e554b8" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoTags" ma:index="11" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="12" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="13" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="14" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="15" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceKeyPoints" ma:index="16" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="18" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Vaizdų žymės" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="993cf2ba-b7a7-49f7-97d1-76e12a88c412" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="23" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="24" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="25" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="aa0d983d-359a-438c-9953-3af1a8ac0831" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="19" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{82c4fa3c-500e-4213-91e5-1b9e2014ea63}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="aa0d983d-359a-438c-9953-3af1a8ac0831">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Bendrinama su" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Bendrinta su išsamia informacija" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Turinio tipas"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Antraštė"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="453e7e53-5eb2-45cf-b2ab-34c867e554b8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="aa0d983d-359a-438c-9953-3af1a8ac0831" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2DEB40B8-8AF4-4C88-8F9E-FB64A82FE8F0}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC542CFB-1FD9-432C-86E5-B15DDE8B6777}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{431465D1-10D6-47A7-B207-6D8BB8936332}"/>
 </file>
</xml_diff>

<commit_message>
Duomenys perkeliami į lapa Greitis su Pradiniai2Funkcija.py
</commit_message>
<xml_diff>
--- a/Rezultatai.xlsx
+++ b/Rezultatai.xlsx
@@ -228,7 +228,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -274,12 +274,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -921,124 +930,166 @@
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>AAA</t>
-        </is>
-      </c>
-      <c r="D6" s="19" t="n">
-        <v>16</v>
-      </c>
-      <c r="E6" s="20" t="n"/>
-      <c r="F6" s="20" t="n"/>
-      <c r="G6" s="20" t="n"/>
-      <c r="H6" s="20" t="n"/>
-      <c r="I6" s="20" t="n"/>
-      <c r="J6" s="21" t="n">
+          <t>Ekopartneris</t>
+        </is>
+      </c>
+      <c r="D6" s="20" t="n">
+        <v>13</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="H6" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="I6" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J6" s="22" t="n">
         <v>0.827</v>
       </c>
-      <c r="K6" s="20" t="n"/>
-      <c r="L6" s="20" t="n"/>
-      <c r="M6" s="20" t="n"/>
-      <c r="N6" s="22" t="n"/>
-      <c r="O6" s="22" t="n"/>
-      <c r="P6" s="22" t="n"/>
-      <c r="Q6" s="22" t="n"/>
-      <c r="R6" s="22" t="n"/>
-      <c r="S6" s="22" t="n"/>
-      <c r="T6" s="22" t="n"/>
-      <c r="U6" s="22" t="n"/>
-      <c r="V6" s="20" t="n"/>
-      <c r="W6" s="22" t="n"/>
-      <c r="X6" s="22" t="n"/>
-      <c r="Y6" s="20" t="n"/>
-      <c r="Z6" s="20" t="n"/>
-      <c r="AA6" s="22" t="n"/>
-      <c r="AB6" s="20" t="n"/>
-      <c r="AC6" s="20" t="n"/>
-      <c r="AD6" s="21" t="n">
+      <c r="K6" s="23" t="n"/>
+      <c r="L6" s="24" t="n">
+        <v>1012</v>
+      </c>
+      <c r="M6" s="24" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="N6" s="25" t="n"/>
+      <c r="O6" s="25" t="n"/>
+      <c r="P6" s="25" t="n"/>
+      <c r="Q6" s="25" t="n"/>
+      <c r="R6" s="25" t="n"/>
+      <c r="S6" s="25" t="n"/>
+      <c r="T6" s="25" t="n"/>
+      <c r="U6" s="25" t="n"/>
+      <c r="V6" s="23" t="n"/>
+      <c r="W6" s="25" t="n"/>
+      <c r="X6" s="25" t="n"/>
+      <c r="Y6" s="23" t="n"/>
+      <c r="Z6" s="23" t="n"/>
+      <c r="AA6" s="25" t="n"/>
+      <c r="AB6" s="23" t="n"/>
+      <c r="AC6" s="23" t="n"/>
+      <c r="AD6" s="22" t="n">
         <v>0.079</v>
       </c>
-      <c r="AE6" s="22" t="n"/>
-      <c r="AF6" s="22" t="n"/>
-      <c r="AG6" s="20" t="n"/>
+      <c r="AE6" s="25" t="n"/>
+      <c r="AF6" s="25" t="n"/>
+      <c r="AG6" s="23" t="n"/>
       <c r="AH6" s="13" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="n"/>
       <c r="B7" s="15" t="n"/>
       <c r="C7" s="15" t="n"/>
-      <c r="D7" s="19" t="n">
-        <v>47</v>
-      </c>
-      <c r="E7" s="20" t="n"/>
-      <c r="F7" s="20" t="n"/>
-      <c r="G7" s="20" t="n"/>
-      <c r="H7" s="20" t="n"/>
-      <c r="I7" s="20" t="n"/>
-      <c r="J7" s="21" t="n">
+      <c r="D7" s="20" t="n">
+        <v>69</v>
+      </c>
+      <c r="E7" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="I7" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J7" s="22" t="n">
         <v>0.827</v>
       </c>
-      <c r="K7" s="20" t="n"/>
-      <c r="L7" s="20" t="n"/>
-      <c r="M7" s="20" t="n"/>
-      <c r="N7" s="22" t="n"/>
-      <c r="O7" s="22" t="n"/>
-      <c r="P7" s="22" t="n"/>
-      <c r="Q7" s="22" t="n"/>
-      <c r="R7" s="22" t="n"/>
-      <c r="S7" s="22" t="n"/>
-      <c r="T7" s="22" t="n"/>
+      <c r="K7" s="23" t="n"/>
+      <c r="L7" s="24" t="n">
+        <v>1012</v>
+      </c>
+      <c r="M7" s="24" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="N7" s="25" t="n"/>
+      <c r="O7" s="25" t="n"/>
+      <c r="P7" s="25" t="n"/>
+      <c r="Q7" s="25" t="n"/>
+      <c r="R7" s="25" t="n"/>
+      <c r="S7" s="25" t="n"/>
+      <c r="T7" s="25" t="n"/>
       <c r="U7" s="13" t="n"/>
-      <c r="V7" s="19" t="inlineStr">
-        <is>
-          <t>1,25</t>
-        </is>
-      </c>
-      <c r="W7" s="23">
+      <c r="V7" s="20" t="inlineStr">
+        <is>
+          <t>1,89</t>
+        </is>
+      </c>
+      <c r="W7" s="26">
         <f>V7*V8</f>
         <v/>
       </c>
-      <c r="X7" s="22" t="n"/>
-      <c r="Y7" s="20" t="n"/>
-      <c r="Z7" s="20" t="n"/>
-      <c r="AA7" s="22" t="n"/>
-      <c r="AB7" s="20" t="n"/>
-      <c r="AC7" s="20" t="n"/>
-      <c r="AD7" s="21" t="n">
+      <c r="X7" s="25" t="n"/>
+      <c r="Y7" s="23" t="n"/>
+      <c r="Z7" s="23" t="n"/>
+      <c r="AA7" s="25" t="n"/>
+      <c r="AB7" s="23" t="n"/>
+      <c r="AC7" s="23" t="n"/>
+      <c r="AD7" s="22" t="n">
         <v>0.079</v>
       </c>
-      <c r="AE7" s="22" t="n"/>
-      <c r="AF7" s="22" t="n"/>
+      <c r="AE7" s="25" t="n"/>
+      <c r="AF7" s="25" t="n"/>
       <c r="AH7" s="16" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="n"/>
       <c r="B8" s="15" t="n"/>
       <c r="C8" s="15" t="n"/>
-      <c r="D8" s="19" t="n">
-        <v>78</v>
-      </c>
-      <c r="E8" s="20" t="n"/>
-      <c r="F8" s="20" t="n"/>
-      <c r="G8" s="20" t="n"/>
-      <c r="H8" s="20" t="n"/>
-      <c r="I8" s="20" t="n"/>
-      <c r="J8" s="21" t="n">
+      <c r="D8" s="20" t="n">
+        <v>116</v>
+      </c>
+      <c r="E8" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="I8" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J8" s="22" t="n">
         <v>0.827</v>
       </c>
-      <c r="K8" s="20" t="n"/>
-      <c r="L8" s="20" t="n"/>
-      <c r="M8" s="20" t="n"/>
-      <c r="N8" s="22" t="n"/>
-      <c r="O8" s="22" t="n"/>
-      <c r="P8" s="22" t="n"/>
-      <c r="Q8" s="22" t="n"/>
-      <c r="R8" s="22" t="n"/>
-      <c r="S8" s="22" t="n"/>
-      <c r="T8" s="22" t="n"/>
+      <c r="K8" s="23" t="n"/>
+      <c r="L8" s="24" t="n">
+        <v>1012</v>
+      </c>
+      <c r="M8" s="24" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="N8" s="25" t="n"/>
+      <c r="O8" s="25" t="n"/>
+      <c r="P8" s="25" t="n"/>
+      <c r="Q8" s="25" t="n"/>
+      <c r="R8" s="25" t="n"/>
+      <c r="S8" s="25" t="n"/>
+      <c r="T8" s="25" t="n"/>
       <c r="U8" s="13" t="n"/>
-      <c r="V8" s="19" t="inlineStr">
-        <is>
-          <t>1,25</t>
+      <c r="V8" s="20" t="inlineStr">
+        <is>
+          <t>1,91</t>
         </is>
       </c>
       <c r="W8" s="13" t="n"/>
@@ -1049,27 +1100,41 @@
       <c r="A9" s="16" t="n"/>
       <c r="B9" s="16" t="n"/>
       <c r="C9" s="16" t="n"/>
-      <c r="D9" s="19" t="n">
-        <v>109</v>
-      </c>
-      <c r="E9" s="20" t="n"/>
-      <c r="F9" s="20" t="n"/>
-      <c r="G9" s="20" t="n"/>
-      <c r="H9" s="20" t="n"/>
-      <c r="I9" s="20" t="n"/>
-      <c r="J9" s="21" t="n">
+      <c r="D9" s="20" t="n">
+        <v>162</v>
+      </c>
+      <c r="E9" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="H9" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="I9" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J9" s="22" t="n">
         <v>0.827</v>
       </c>
-      <c r="K9" s="20" t="n"/>
-      <c r="L9" s="20" t="n"/>
-      <c r="M9" s="20" t="n"/>
-      <c r="N9" s="22" t="n"/>
-      <c r="O9" s="22" t="n"/>
-      <c r="P9" s="22" t="n"/>
-      <c r="Q9" s="22" t="n"/>
-      <c r="R9" s="22" t="n"/>
-      <c r="S9" s="22" t="n"/>
-      <c r="T9" s="22" t="n"/>
+      <c r="K9" s="23" t="n"/>
+      <c r="L9" s="24" t="n">
+        <v>1012</v>
+      </c>
+      <c r="M9" s="24" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="N9" s="25" t="n"/>
+      <c r="O9" s="25" t="n"/>
+      <c r="P9" s="25" t="n"/>
+      <c r="Q9" s="25" t="n"/>
+      <c r="R9" s="25" t="n"/>
+      <c r="S9" s="25" t="n"/>
+      <c r="T9" s="25" t="n"/>
       <c r="U9" s="13" t="n"/>
       <c r="V9" s="13" t="n"/>
       <c r="W9" s="13" t="n"/>
@@ -1102,12 +1167,12 @@
       <c r="A11" s="13" t="n"/>
       <c r="B11" s="13" t="n"/>
       <c r="C11" s="13" t="n"/>
-      <c r="D11" s="24" t="inlineStr">
+      <c r="D11" s="27" t="inlineStr">
         <is>
           <t>RPU***</t>
         </is>
       </c>
-      <c r="E11" s="25" t="inlineStr">
+      <c r="E11" s="28" t="inlineStr">
         <is>
           <t>Kai bus 2 linijos, RPU*** yra 2 linijos vidurinis taškas</t>
         </is>
@@ -1441,12 +1506,12 @@
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>AAA</t>
+          <t>Ekopartneris</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>1,25 x 1,25</t>
+          <t>1,89 x 1,91</t>
         </is>
       </c>
       <c r="E6" s="11">
@@ -1595,7 +1660,7 @@
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>AAA</t>
+          <t>Ekopartneris</t>
         </is>
       </c>
     </row>
@@ -1742,78 +1807,78 @@
       </c>
     </row>
     <row r="6" ht="25" customHeight="1">
-      <c r="A6" s="34" t="inlineStr">
+      <c r="A6" s="37" t="inlineStr">
         <is>
           <t>2026-02-10</t>
         </is>
       </c>
-      <c r="B6" s="34" t="n">
+      <c r="B6" s="37" t="n">
         <v>5</v>
       </c>
-      <c r="C6" s="27" t="inlineStr">
-        <is>
-          <t>AAA</t>
-        </is>
-      </c>
-      <c r="D6" s="28" t="n"/>
-      <c r="E6" s="29" t="n"/>
-      <c r="F6" s="29" t="n"/>
-      <c r="G6" s="29" t="n"/>
-      <c r="H6" s="29" t="n"/>
-      <c r="I6" s="29" t="n"/>
-      <c r="J6" s="29" t="n"/>
-      <c r="K6" s="29" t="n"/>
-      <c r="L6" s="30" t="n"/>
-      <c r="M6" s="30" t="n"/>
-      <c r="N6" s="27" t="n"/>
-      <c r="O6" s="27" t="n">
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>Ekopartneris</t>
+        </is>
+      </c>
+      <c r="D6" s="31" t="n"/>
+      <c r="E6" s="32" t="n"/>
+      <c r="F6" s="32" t="n"/>
+      <c r="G6" s="32" t="n"/>
+      <c r="H6" s="32" t="n"/>
+      <c r="I6" s="32" t="n"/>
+      <c r="J6" s="32" t="n"/>
+      <c r="K6" s="32" t="n"/>
+      <c r="L6" s="33" t="n"/>
+      <c r="M6" s="33" t="n"/>
+      <c r="N6" s="30" t="n"/>
+      <c r="O6" s="30" t="n">
         <v>3</v>
       </c>
-      <c r="P6" s="31" t="inlineStr">
+      <c r="P6" s="34" t="inlineStr">
         <is>
           <t>5 linijos, 1 filtras</t>
         </is>
       </c>
     </row>
     <row r="7" ht="25" customHeight="1">
-      <c r="A7" s="35" t="n"/>
-      <c r="B7" s="35" t="n"/>
-      <c r="C7" s="35" t="n"/>
-      <c r="D7" s="28" t="n"/>
-      <c r="E7" s="29" t="n"/>
-      <c r="F7" s="29" t="n"/>
-      <c r="G7" s="29" t="n"/>
-      <c r="H7" s="29" t="n"/>
-      <c r="I7" s="29" t="n"/>
-      <c r="J7" s="29" t="n"/>
-      <c r="K7" s="29" t="n"/>
-      <c r="L7" s="35" t="n"/>
-      <c r="M7" s="35" t="n"/>
-      <c r="N7" s="35" t="n"/>
-      <c r="O7" s="35" t="n"/>
-      <c r="P7" s="31" t="inlineStr">
+      <c r="A7" s="38" t="n"/>
+      <c r="B7" s="38" t="n"/>
+      <c r="C7" s="38" t="n"/>
+      <c r="D7" s="31" t="n"/>
+      <c r="E7" s="32" t="n"/>
+      <c r="F7" s="32" t="n"/>
+      <c r="G7" s="32" t="n"/>
+      <c r="H7" s="32" t="n"/>
+      <c r="I7" s="32" t="n"/>
+      <c r="J7" s="32" t="n"/>
+      <c r="K7" s="32" t="n"/>
+      <c r="L7" s="38" t="n"/>
+      <c r="M7" s="38" t="n"/>
+      <c r="N7" s="38" t="n"/>
+      <c r="O7" s="38" t="n"/>
+      <c r="P7" s="34" t="inlineStr">
         <is>
           <t>5 linijos, 2 filtras</t>
         </is>
       </c>
     </row>
     <row r="8" ht="25" customHeight="1">
-      <c r="A8" s="36" t="n"/>
-      <c r="B8" s="36" t="n"/>
-      <c r="C8" s="36" t="n"/>
-      <c r="D8" s="28" t="n"/>
-      <c r="E8" s="29" t="n"/>
-      <c r="F8" s="29" t="n"/>
-      <c r="G8" s="29" t="n"/>
-      <c r="H8" s="29" t="n"/>
-      <c r="I8" s="29" t="n"/>
-      <c r="J8" s="29" t="n"/>
-      <c r="K8" s="29" t="n"/>
-      <c r="L8" s="36" t="n"/>
-      <c r="M8" s="36" t="n"/>
-      <c r="N8" s="36" t="n"/>
-      <c r="O8" s="36" t="n"/>
-      <c r="P8" s="31" t="inlineStr">
+      <c r="A8" s="39" t="n"/>
+      <c r="B8" s="39" t="n"/>
+      <c r="C8" s="39" t="n"/>
+      <c r="D8" s="31" t="n"/>
+      <c r="E8" s="32" t="n"/>
+      <c r="F8" s="32" t="n"/>
+      <c r="G8" s="32" t="n"/>
+      <c r="H8" s="32" t="n"/>
+      <c r="I8" s="32" t="n"/>
+      <c r="J8" s="32" t="n"/>
+      <c r="K8" s="32" t="n"/>
+      <c r="L8" s="39" t="n"/>
+      <c r="M8" s="39" t="n"/>
+      <c r="N8" s="39" t="n"/>
+      <c r="O8" s="39" t="n"/>
+      <c r="P8" s="34" t="inlineStr">
         <is>
           <t>5 linijos, 3 filtras</t>
         </is>
@@ -1970,255 +2035,255 @@
       <c r="O5" s="16" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="37" t="n">
+      <c r="A6" s="40" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="37" t="inlineStr">
-        <is>
-          <t>AAA</t>
-        </is>
-      </c>
-      <c r="C6" s="38" t="n">
+      <c r="B6" s="40" t="inlineStr">
+        <is>
+          <t>Ekopartneris</t>
+        </is>
+      </c>
+      <c r="C6" s="41" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="39" t="n"/>
-      <c r="E6" s="20" t="n"/>
-      <c r="F6" s="20" t="n"/>
-      <c r="G6" s="20" t="n"/>
-      <c r="H6" s="39" t="n"/>
-      <c r="I6" s="39" t="n"/>
-      <c r="J6" s="20" t="n"/>
-      <c r="K6" s="20" t="n"/>
-      <c r="L6" s="20" t="n"/>
-      <c r="M6" s="22" t="n"/>
-      <c r="N6" s="39" t="n"/>
-      <c r="O6" s="40" t="inlineStr">
+      <c r="D6" s="42" t="n"/>
+      <c r="E6" s="23" t="n"/>
+      <c r="F6" s="23" t="n"/>
+      <c r="G6" s="23" t="n"/>
+      <c r="H6" s="42" t="n"/>
+      <c r="I6" s="42" t="n"/>
+      <c r="J6" s="23" t="n"/>
+      <c r="K6" s="23" t="n"/>
+      <c r="L6" s="23" t="n"/>
+      <c r="M6" s="25" t="n"/>
+      <c r="N6" s="42" t="n"/>
+      <c r="O6" s="43" t="inlineStr">
         <is>
           <t>5 linijos, 3 filtrai</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="41" t="n"/>
-      <c r="B7" s="41" t="n"/>
-      <c r="C7" s="38" t="n">
+      <c r="A7" s="44" t="n"/>
+      <c r="B7" s="44" t="n"/>
+      <c r="C7" s="41" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="41" t="n"/>
-      <c r="E7" s="20" t="n"/>
-      <c r="F7" s="20" t="n"/>
-      <c r="G7" s="20" t="n"/>
-      <c r="H7" s="41" t="n"/>
-      <c r="I7" s="41" t="n"/>
-      <c r="J7" s="20" t="n"/>
-      <c r="K7" s="20" t="n"/>
-      <c r="L7" s="20" t="n"/>
-      <c r="M7" s="22" t="n"/>
-      <c r="N7" s="41" t="n"/>
+      <c r="D7" s="44" t="n"/>
+      <c r="E7" s="23" t="n"/>
+      <c r="F7" s="23" t="n"/>
+      <c r="G7" s="23" t="n"/>
+      <c r="H7" s="44" t="n"/>
+      <c r="I7" s="44" t="n"/>
+      <c r="J7" s="23" t="n"/>
+      <c r="K7" s="23" t="n"/>
+      <c r="L7" s="23" t="n"/>
+      <c r="M7" s="25" t="n"/>
+      <c r="N7" s="44" t="n"/>
       <c r="O7" s="13" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="41" t="n"/>
-      <c r="B8" s="41" t="n"/>
-      <c r="C8" s="38" t="n">
+      <c r="A8" s="44" t="n"/>
+      <c r="B8" s="44" t="n"/>
+      <c r="C8" s="41" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="41" t="n"/>
-      <c r="E8" s="20" t="n"/>
-      <c r="F8" s="20" t="n"/>
-      <c r="G8" s="20" t="n"/>
-      <c r="H8" s="41" t="n"/>
-      <c r="I8" s="41" t="n"/>
-      <c r="J8" s="20" t="n"/>
-      <c r="K8" s="20" t="n"/>
-      <c r="L8" s="20" t="n"/>
-      <c r="M8" s="22" t="n"/>
-      <c r="N8" s="41" t="n"/>
+      <c r="D8" s="44" t="n"/>
+      <c r="E8" s="23" t="n"/>
+      <c r="F8" s="23" t="n"/>
+      <c r="G8" s="23" t="n"/>
+      <c r="H8" s="44" t="n"/>
+      <c r="I8" s="44" t="n"/>
+      <c r="J8" s="23" t="n"/>
+      <c r="K8" s="23" t="n"/>
+      <c r="L8" s="23" t="n"/>
+      <c r="M8" s="25" t="n"/>
+      <c r="N8" s="44" t="n"/>
       <c r="O8" s="13" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="41" t="n"/>
-      <c r="B9" s="41" t="n"/>
-      <c r="C9" s="38" t="inlineStr">
+      <c r="A9" s="44" t="n"/>
+      <c r="B9" s="44" t="n"/>
+      <c r="C9" s="41" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D9" s="41" t="n"/>
-      <c r="E9" s="20" t="n"/>
-      <c r="F9" s="20" t="n"/>
-      <c r="G9" s="20" t="n"/>
-      <c r="H9" s="41" t="n"/>
-      <c r="I9" s="41" t="n"/>
-      <c r="J9" s="20" t="n"/>
-      <c r="K9" s="20" t="n"/>
-      <c r="L9" s="20" t="n"/>
-      <c r="M9" s="22" t="n"/>
-      <c r="N9" s="41" t="n"/>
-      <c r="O9" s="42" t="inlineStr">
+      <c r="D9" s="44" t="n"/>
+      <c r="E9" s="23" t="n"/>
+      <c r="F9" s="23" t="n"/>
+      <c r="G9" s="23" t="n"/>
+      <c r="H9" s="44" t="n"/>
+      <c r="I9" s="44" t="n"/>
+      <c r="J9" s="23" t="n"/>
+      <c r="K9" s="23" t="n"/>
+      <c r="L9" s="23" t="n"/>
+      <c r="M9" s="25" t="n"/>
+      <c r="N9" s="44" t="n"/>
+      <c r="O9" s="45" t="inlineStr">
         <is>
           <t>Tuščiasis ėminys (mt)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="41" t="n"/>
-      <c r="B10" s="41" t="n"/>
+      <c r="A10" s="44" t="n"/>
+      <c r="B10" s="44" t="n"/>
       <c r="C10" s="13" t="n"/>
-      <c r="D10" s="41" t="n"/>
+      <c r="D10" s="44" t="n"/>
       <c r="E10" s="13" t="n"/>
       <c r="F10" s="13" t="n"/>
       <c r="G10" s="13" t="n"/>
-      <c r="H10" s="41" t="n"/>
-      <c r="I10" s="41" t="n"/>
+      <c r="H10" s="44" t="n"/>
+      <c r="I10" s="44" t="n"/>
       <c r="J10" s="13" t="n"/>
       <c r="K10" s="13" t="n"/>
       <c r="L10" s="13" t="n"/>
       <c r="M10" s="13" t="n"/>
-      <c r="N10" s="41" t="n"/>
+      <c r="N10" s="44" t="n"/>
       <c r="O10" s="13" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="41" t="n"/>
-      <c r="B11" s="41" t="n"/>
-      <c r="C11" s="38" t="inlineStr">
+      <c r="A11" s="44" t="n"/>
+      <c r="B11" s="44" t="n"/>
+      <c r="C11" s="41" t="inlineStr">
         <is>
           <t>41</t>
         </is>
       </c>
-      <c r="D11" s="41" t="n"/>
-      <c r="E11" s="20" t="n"/>
-      <c r="F11" s="20" t="n"/>
-      <c r="G11" s="20" t="n"/>
-      <c r="H11" s="41" t="n"/>
-      <c r="I11" s="41" t="n"/>
-      <c r="J11" s="20" t="n"/>
-      <c r="K11" s="20" t="n"/>
-      <c r="L11" s="20" t="n"/>
-      <c r="M11" s="22" t="n"/>
-      <c r="N11" s="41" t="n"/>
-      <c r="O11" s="42" t="inlineStr">
+      <c r="D11" s="44" t="n"/>
+      <c r="E11" s="23" t="n"/>
+      <c r="F11" s="23" t="n"/>
+      <c r="G11" s="23" t="n"/>
+      <c r="H11" s="44" t="n"/>
+      <c r="I11" s="44" t="n"/>
+      <c r="J11" s="23" t="n"/>
+      <c r="K11" s="23" t="n"/>
+      <c r="L11" s="23" t="n"/>
+      <c r="M11" s="25" t="n"/>
+      <c r="N11" s="44" t="n"/>
+      <c r="O11" s="45" t="inlineStr">
         <is>
           <t>Išplautos nuosėdos (mn)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="41" t="n"/>
-      <c r="B12" s="41" t="n"/>
-      <c r="C12" s="38" t="inlineStr">
+      <c r="A12" s="44" t="n"/>
+      <c r="B12" s="44" t="n"/>
+      <c r="C12" s="41" t="inlineStr">
         <is>
           <t>00</t>
         </is>
       </c>
-      <c r="D12" s="41" t="n"/>
-      <c r="E12" s="20" t="n"/>
-      <c r="F12" s="20" t="n"/>
-      <c r="G12" s="20" t="n"/>
-      <c r="H12" s="41" t="n"/>
-      <c r="I12" s="41" t="n"/>
-      <c r="J12" s="20" t="n"/>
-      <c r="K12" s="20" t="n"/>
-      <c r="L12" s="20" t="n"/>
-      <c r="M12" s="22" t="n"/>
-      <c r="N12" s="41" t="n"/>
-      <c r="O12" s="42" t="inlineStr">
+      <c r="D12" s="44" t="n"/>
+      <c r="E12" s="23" t="n"/>
+      <c r="F12" s="23" t="n"/>
+      <c r="G12" s="23" t="n"/>
+      <c r="H12" s="44" t="n"/>
+      <c r="I12" s="44" t="n"/>
+      <c r="J12" s="23" t="n"/>
+      <c r="K12" s="23" t="n"/>
+      <c r="L12" s="23" t="n"/>
+      <c r="M12" s="25" t="n"/>
+      <c r="N12" s="44" t="n"/>
+      <c r="O12" s="45" t="inlineStr">
         <is>
           <t>Išvalytos ėminių sistemos tuščiasis ėminys (mIt)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="41" t="n"/>
-      <c r="B13" s="41" t="n"/>
-      <c r="C13" s="38" t="inlineStr">
+      <c r="A13" s="44" t="n"/>
+      <c r="B13" s="44" t="n"/>
+      <c r="C13" s="41" t="inlineStr">
         <is>
           <t>01</t>
         </is>
       </c>
-      <c r="D13" s="41" t="n"/>
-      <c r="E13" s="20" t="n"/>
-      <c r="F13" s="20" t="n"/>
-      <c r="G13" s="20" t="n"/>
-      <c r="H13" s="41" t="n"/>
-      <c r="I13" s="41" t="n"/>
-      <c r="J13" s="20" t="n"/>
-      <c r="K13" s="20" t="n"/>
-      <c r="L13" s="20" t="n"/>
-      <c r="M13" s="22" t="n"/>
-      <c r="N13" s="41" t="n"/>
-      <c r="O13" s="42" t="inlineStr">
+      <c r="D13" s="44" t="n"/>
+      <c r="E13" s="23" t="n"/>
+      <c r="F13" s="23" t="n"/>
+      <c r="G13" s="23" t="n"/>
+      <c r="H13" s="44" t="n"/>
+      <c r="I13" s="44" t="n"/>
+      <c r="J13" s="23" t="n"/>
+      <c r="K13" s="23" t="n"/>
+      <c r="L13" s="23" t="n"/>
+      <c r="M13" s="25" t="n"/>
+      <c r="N13" s="44" t="n"/>
+      <c r="O13" s="45" t="inlineStr">
         <is>
           <t>Tušti indai svorio kontrolei (mIt1)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="41" t="n"/>
-      <c r="B14" s="41" t="n"/>
-      <c r="C14" s="38" t="inlineStr">
+      <c r="A14" s="44" t="n"/>
+      <c r="B14" s="44" t="n"/>
+      <c r="C14" s="41" t="inlineStr">
         <is>
           <t>02</t>
         </is>
       </c>
-      <c r="D14" s="41" t="n"/>
-      <c r="E14" s="20" t="n"/>
-      <c r="F14" s="20" t="n"/>
-      <c r="G14" s="20" t="n"/>
-      <c r="H14" s="41" t="n"/>
-      <c r="I14" s="41" t="n"/>
-      <c r="J14" s="20" t="n"/>
-      <c r="K14" s="20" t="n"/>
-      <c r="L14" s="20" t="n"/>
-      <c r="M14" s="22" t="n"/>
-      <c r="N14" s="41" t="n"/>
-      <c r="O14" s="42" t="inlineStr">
+      <c r="D14" s="44" t="n"/>
+      <c r="E14" s="23" t="n"/>
+      <c r="F14" s="23" t="n"/>
+      <c r="G14" s="23" t="n"/>
+      <c r="H14" s="44" t="n"/>
+      <c r="I14" s="44" t="n"/>
+      <c r="J14" s="23" t="n"/>
+      <c r="K14" s="23" t="n"/>
+      <c r="L14" s="23" t="n"/>
+      <c r="M14" s="25" t="n"/>
+      <c r="N14" s="44" t="n"/>
+      <c r="O14" s="45" t="inlineStr">
         <is>
           <t>Tušti indai svorio kontrolei (mIt2)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="41" t="n"/>
-      <c r="B15" s="41" t="n"/>
-      <c r="C15" s="38" t="inlineStr">
+      <c r="A15" s="44" t="n"/>
+      <c r="B15" s="44" t="n"/>
+      <c r="C15" s="41" t="inlineStr">
         <is>
           <t>03</t>
         </is>
       </c>
-      <c r="D15" s="41" t="n"/>
-      <c r="E15" s="20" t="n"/>
-      <c r="F15" s="20" t="n"/>
-      <c r="G15" s="20" t="n"/>
-      <c r="H15" s="41" t="n"/>
-      <c r="I15" s="41" t="n"/>
-      <c r="J15" s="20" t="n"/>
-      <c r="K15" s="20" t="n"/>
-      <c r="L15" s="20" t="n"/>
-      <c r="M15" s="22" t="n"/>
-      <c r="N15" s="41" t="n"/>
-      <c r="O15" s="42" t="inlineStr">
+      <c r="D15" s="44" t="n"/>
+      <c r="E15" s="23" t="n"/>
+      <c r="F15" s="23" t="n"/>
+      <c r="G15" s="23" t="n"/>
+      <c r="H15" s="44" t="n"/>
+      <c r="I15" s="44" t="n"/>
+      <c r="J15" s="23" t="n"/>
+      <c r="K15" s="23" t="n"/>
+      <c r="L15" s="23" t="n"/>
+      <c r="M15" s="25" t="n"/>
+      <c r="N15" s="44" t="n"/>
+      <c r="O15" s="45" t="inlineStr">
         <is>
           <t>Tušti indai svorio kontrolei (mIt3)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="43" t="n"/>
-      <c r="B16" s="43" t="n"/>
+      <c r="A16" s="46" t="n"/>
+      <c r="B16" s="46" t="n"/>
       <c r="C16" s="13" t="n"/>
-      <c r="D16" s="43" t="n"/>
+      <c r="D16" s="46" t="n"/>
       <c r="E16" s="13" t="n"/>
       <c r="F16" s="13" t="n"/>
       <c r="G16" s="13" t="n"/>
-      <c r="H16" s="43" t="n"/>
-      <c r="I16" s="43" t="n"/>
+      <c r="H16" s="46" t="n"/>
+      <c r="I16" s="46" t="n"/>
       <c r="J16" s="13" t="n"/>
       <c r="K16" s="13" t="n"/>
       <c r="L16" s="13" t="n"/>
-      <c r="M16" s="22" t="n"/>
-      <c r="N16" s="43" t="n"/>
-      <c r="O16" s="42" t="inlineStr">
+      <c r="M16" s="25" t="n"/>
+      <c r="N16" s="46" t="n"/>
+      <c r="O16" s="45" t="inlineStr">
         <is>
           <t>Tuščių indų ir išvalytos ėminių sistemos tuščiojo ėminio svorio pokytis (mItp)</t>
         </is>

</xml_diff>